<commit_message>
feat: Add 009821 Nomura Global Rare Earth ETF to passive comparison list (市值型 sheet)
</commit_message>
<xml_diff>
--- a/wiki/金融投資/台灣ETF比較清單.xlsx
+++ b/wiki/金融投資/台灣ETF比較清單.xlsx
@@ -1714,7 +1714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2662,6 +2662,53 @@
         </is>
       </c>
       <c r="I20" t="inlineStr">
+        <is>
+          <t>不配息</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>009821</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>野村全球稀土與關鍵資源</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>張怡琳</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>永豐商業銀行</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>NYSE TIP全球稀土與關鍵資源指數</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>不配息</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.90%</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>0.20%</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>不配息</t>
         </is>

</xml_diff>

<commit_message>
20260902 主動型 ETF 持股日更（第 71 次）：30 檔 1817 筆，每日個股合計 52541 列，dashboard_data.js 更新至 20260902
</commit_message>
<xml_diff>
--- a/wiki/金融投資/台灣ETF比較清單.xlsx
+++ b/wiki/金融投資/台灣ETF比較清單.xlsx
@@ -511,7 +511,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>00400A</t>
         </is>
@@ -553,7 +553,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>00401A</t>
         </is>
@@ -595,7 +595,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>00402A</t>
         </is>
@@ -637,7 +637,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>00403A</t>
         </is>
@@ -679,7 +679,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>00404A</t>
         </is>
@@ -721,7 +721,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>00405A</t>
         </is>
@@ -763,7 +763,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>00407A</t>
         </is>
@@ -805,7 +805,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>00408A</t>
         </is>
@@ -847,7 +847,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>00980A</t>
         </is>
@@ -889,7 +889,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>00981A</t>
         </is>
@@ -931,7 +931,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>00982A</t>
         </is>
@@ -973,7 +973,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>00983A</t>
         </is>
@@ -1015,7 +1015,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>00984A</t>
         </is>
@@ -1057,7 +1057,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>00985A</t>
         </is>
@@ -1099,7 +1099,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>00986A</t>
         </is>
@@ -1141,7 +1141,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>00987A</t>
         </is>
@@ -1183,7 +1183,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>00988A</t>
         </is>
@@ -1225,7 +1225,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>00989A</t>
         </is>
@@ -1267,7 +1267,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>00990A</t>
         </is>
@@ -1309,7 +1309,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>00991A</t>
         </is>
@@ -1351,7 +1351,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>00992A</t>
         </is>
@@ -1393,7 +1393,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>00993A</t>
         </is>
@@ -1435,7 +1435,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>00994A</t>
         </is>
@@ -1477,7 +1477,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>00995A</t>
         </is>
@@ -1519,7 +1519,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>00996A</t>
         </is>
@@ -1561,7 +1561,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>00997A</t>
         </is>
@@ -1603,7 +1603,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>00998A</t>
         </is>
@@ -1645,7 +1645,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>00999A</t>
         </is>
@@ -1687,7 +1687,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>00980D</t>
         </is>
@@ -1729,7 +1729,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>00983D</t>
         </is>
@@ -1772,38 +1772,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H33"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId30"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>

</xml_diff>